<commit_message>
progress: 49 village workbooks (randomwalk-TRX50-WS 2026-10-10T02:50:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Enathimelpakkam_13.398667_80.153513.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Enathimelpakkam_13.398667_80.153513.xlsx
@@ -2666,6 +2666,11 @@
           <t>269</t>
         </is>
       </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -2673,6 +2678,11 @@
           <t>27</t>
         </is>
       </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -2680,6 +2690,11 @@
           <t>270</t>
         </is>
       </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -2687,6 +2702,11 @@
           <t>271</t>
         </is>
       </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -2694,6 +2714,11 @@
           <t>272</t>
         </is>
       </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -2701,6 +2726,11 @@
           <t>273</t>
         </is>
       </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -2708,6 +2738,11 @@
           <t>274</t>
         </is>
       </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -2715,6 +2750,11 @@
           <t>275</t>
         </is>
       </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>1, 2, 3A1, 3A2, 3B, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -2722,6 +2762,11 @@
           <t>276</t>
         </is>
       </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -2729,6 +2774,11 @@
           <t>277</t>
         </is>
       </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -2736,6 +2786,11 @@
           <t>278</t>
         </is>
       </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -2743,6 +2798,11 @@
           <t>279</t>
         </is>
       </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B1, 2B2, 3, 4, 5, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -2750,6 +2810,11 @@
           <t>28</t>
         </is>
       </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B, 5A, 5B</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -2757,6 +2822,11 @@
           <t>280</t>
         </is>
       </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -2764,6 +2834,11 @@
           <t>281</t>
         </is>
       </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 1A1A, 1B, 20, 21A, 21B, 22, 23, 24, 25, 26, 27, 28, 29, 2A, 3, 30, 31, 32, 33, 34, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -2771,6 +2846,11 @@
           <t>282</t>
         </is>
       </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15A, 15B, 16, 17, 18, 19, 2, 20, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -2778,6 +2858,11 @@
           <t>283</t>
         </is>
       </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -2785,6 +2870,11 @@
           <t>284</t>
         </is>
       </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -2792,6 +2882,11 @@
           <t>285</t>
         </is>
       </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>1, 10, 2A1A1A, 2A2, 2B, 3, 4A, 4B, 5A, 5B, 6A, 6B, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -2799,6 +2894,11 @@
           <t>286</t>
         </is>
       </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -2806,6 +2906,11 @@
           <t>287</t>
         </is>
       </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -2813,6 +2918,11 @@
           <t>288</t>
         </is>
       </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5A, 5B, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -2820,6 +2930,11 @@
           <t>289</t>
         </is>
       </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -2827,6 +2942,11 @@
           <t>29</t>
         </is>
       </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 4, 5A, 5B, 6A, 6B</t>
+        </is>
+      </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -2834,6 +2954,11 @@
           <t>290</t>
         </is>
       </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -2841,6 +2966,11 @@
           <t>291</t>
         </is>
       </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -2848,6 +2978,11 @@
           <t>292</t>
         </is>
       </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -2855,6 +2990,11 @@
           <t>293</t>
         </is>
       </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -2862,6 +3002,11 @@
           <t>294</t>
         </is>
       </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -2869,6 +3014,11 @@
           <t>295</t>
         </is>
       </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 2, 3, 4A, 4B, 5, 6A, 6B, 7, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -2876,6 +3026,11 @@
           <t>296</t>
         </is>
       </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -2883,6 +3038,11 @@
           <t>297</t>
         </is>
       </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -2890,6 +3050,11 @@
           <t>298</t>
         </is>
       </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -2897,6 +3062,11 @@
           <t>299</t>
         </is>
       </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -2904,6 +3074,11 @@
           <t>3</t>
         </is>
       </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -2911,6 +3086,11 @@
           <t>30</t>
         </is>
       </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -2918,6 +3098,11 @@
           <t>300</t>
         </is>
       </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -2925,6 +3110,11 @@
           <t>301</t>
         </is>
       </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -2932,6 +3122,11 @@
           <t>302</t>
         </is>
       </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -2939,6 +3134,11 @@
           <t>303</t>
         </is>
       </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -2946,6 +3146,11 @@
           <t>304</t>
         </is>
       </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -2953,6 +3158,11 @@
           <t>305</t>
         </is>
       </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -2960,6 +3170,11 @@
           <t>306</t>
         </is>
       </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -2967,6 +3182,11 @@
           <t>307</t>
         </is>
       </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -2974,6 +3194,11 @@
           <t>308</t>
         </is>
       </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -2981,6 +3206,11 @@
           <t>309</t>
         </is>
       </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -2988,6 +3218,11 @@
           <t>31</t>
         </is>
       </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2B, 2C, 3A1, 3B, 3C, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -2995,6 +3230,11 @@
           <t>310</t>
         </is>
       </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A1, 2A2, 2B1, 2B2, 2C</t>
+        </is>
+      </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -3002,6 +3242,11 @@
           <t>311</t>
         </is>
       </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -3009,6 +3254,11 @@
           <t>312</t>
         </is>
       </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3A, 3B, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -3016,6 +3266,11 @@
           <t>313</t>
         </is>
       </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
@@ -3023,6 +3278,11 @@
           <t>314</t>
         </is>
       </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
@@ -3030,6 +3290,11 @@
           <t>315</t>
         </is>
       </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
@@ -3037,6 +3302,11 @@
           <t>316</t>
         </is>
       </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 2, 3, 4, 5A, 5B, 6A, 6B, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -3044,6 +3314,11 @@
           <t>317</t>
         </is>
       </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14A, 14B, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -3051,6 +3326,11 @@
           <t>318</t>
         </is>
       </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -3058,6 +3338,11 @@
           <t>319</t>
         </is>
       </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2A1, 2A2, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
@@ -3065,6 +3350,11 @@
           <t>32</t>
         </is>
       </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7, 8, 9A1, 9A2, 9B, 9C</t>
+        </is>
+      </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -3072,6 +3362,11 @@
           <t>320</t>
         </is>
       </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3A, 3B, 3C, 4A, 4B, 5, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
@@ -3079,6 +3374,11 @@
           <t>321</t>
         </is>
       </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -3086,6 +3386,11 @@
           <t>322</t>
         </is>
       </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -3093,6 +3398,11 @@
           <t>33</t>
         </is>
       </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
@@ -3100,6 +3410,11 @@
           <t>34</t>
         </is>
       </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -3107,6 +3422,11 @@
           <t>35</t>
         </is>
       </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
@@ -3114,6 +3434,11 @@
           <t>36</t>
         </is>
       </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
@@ -3121,6 +3446,11 @@
           <t>37</t>
         </is>
       </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
@@ -3128,6 +3458,11 @@
           <t>38</t>
         </is>
       </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
@@ -3135,6 +3470,11 @@
           <t>39</t>
         </is>
       </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15A, 15B, 16, 17, 18A, 18B, 19, 20A, 20B, 21A1A, 21A2, 21B1, 21B2, 21B3, 21B4, 22A1A, 22A2A, 22A3, 22B1, 22B2, 22B3, 22B4, 22B5, 22B6, 22B7, 23, 24, 25, 26, 27, 2A, 2B, 3A, 3B, 4, 5, 6, 7, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
@@ -3142,6 +3482,11 @@
           <t>4</t>
         </is>
       </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
@@ -3149,6 +3494,11 @@
           <t>40A</t>
         </is>
       </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2A, 2B, 2C</t>
+        </is>
+      </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
@@ -3156,6 +3506,11 @@
           <t>40B</t>
         </is>
       </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B1, 1B2, 2A1, 2A2, 2A3, 2B, 3, 4A1, 4A2, 4A3, 4A4, 4A5, 4A6, 4B, 5A, 5B, 5C, 6</t>
+        </is>
+      </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
@@ -3163,6 +3518,11 @@
           <t>41</t>
         </is>
       </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A1, 2A2, 2A3, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
@@ -3170,6 +3530,11 @@
           <t>42</t>
         </is>
       </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
@@ -3177,6 +3542,11 @@
           <t>43</t>
         </is>
       </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
@@ -3184,6 +3554,11 @@
           <t>44</t>
         </is>
       </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -3191,6 +3566,11 @@
           <t>45</t>
         </is>
       </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
@@ -3198,6 +3578,11 @@
           <t>46</t>
         </is>
       </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
@@ -3205,6 +3590,11 @@
           <t>47</t>
         </is>
       </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 4, 5, 6A, 6B, 7</t>
+        </is>
+      </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
@@ -3212,6 +3602,11 @@
           <t>48</t>
         </is>
       </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
@@ -3219,6 +3614,11 @@
           <t>49</t>
         </is>
       </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 2A, 2B, 2C, 2D, 3</t>
+        </is>
+      </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
@@ -3226,6 +3626,11 @@
           <t>5</t>
         </is>
       </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
@@ -3233,6 +3638,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7, 8, 9A, 9B1, 9B2</t>
+        </is>
+      </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
@@ -3240,6 +3650,11 @@
           <t>51</t>
         </is>
       </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
@@ -3247,6 +3662,11 @@
           <t>52</t>
         </is>
       </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
@@ -3254,6 +3674,11 @@
           <t>53</t>
         </is>
       </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
@@ -3261,6 +3686,11 @@
           <t>54</t>
         </is>
       </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
@@ -3268,6 +3698,11 @@
           <t>55</t>
         </is>
       </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
@@ -3275,6 +3710,11 @@
           <t>56</t>
         </is>
       </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C</t>
+        </is>
+      </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
@@ -3282,6 +3722,11 @@
           <t>57</t>
         </is>
       </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>1, 2, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
@@ -3289,6 +3734,11 @@
           <t>58</t>
         </is>
       </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
@@ -3296,6 +3746,11 @@
           <t>59</t>
         </is>
       </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
@@ -3303,11 +3758,21 @@
           <t>6</t>
         </is>
       </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
           <t>60</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>1, 2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 51 village workbooks (randomwalk-TRX50-WS 2026-10-10T03:00:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Enathimelpakkam_13.398667_80.153513.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Enathimelpakkam_13.398667_80.153513.xlsx
@@ -3782,6 +3782,11 @@
           <t>61</t>
         </is>
       </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
@@ -3789,6 +3794,11 @@
           <t>62</t>
         </is>
       </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
@@ -3796,6 +3806,11 @@
           <t>63</t>
         </is>
       </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
@@ -3803,6 +3818,11 @@
           <t>64</t>
         </is>
       </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
@@ -3810,6 +3830,11 @@
           <t>65</t>
         </is>
       </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
@@ -3817,6 +3842,11 @@
           <t>66</t>
         </is>
       </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
@@ -3824,6 +3854,11 @@
           <t>67</t>
         </is>
       </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
@@ -3831,6 +3866,11 @@
           <t>68</t>
         </is>
       </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
@@ -3838,6 +3878,11 @@
           <t>69</t>
         </is>
       </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
@@ -3845,6 +3890,11 @@
           <t>7</t>
         </is>
       </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
@@ -3852,6 +3902,11 @@
           <t>70</t>
         </is>
       </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
@@ -3859,6 +3914,11 @@
           <t>71</t>
         </is>
       </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 3C, 3D1, 3D2, 3D3, 4, 5, 6A1, 6A2, 6B1, 6B2, 6B3, 6B4, 6B5, 6B6</t>
+        </is>
+      </c>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
@@ -3866,6 +3926,11 @@
           <t>72</t>
         </is>
       </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
@@ -3873,6 +3938,11 @@
           <t>73</t>
         </is>
       </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
@@ -3880,6 +3950,11 @@
           <t>74</t>
         </is>
       </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
@@ -3887,6 +3962,11 @@
           <t>75</t>
         </is>
       </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3A, 3B, 4</t>
+        </is>
+      </c>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
@@ -3894,6 +3974,11 @@
           <t>76</t>
         </is>
       </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
@@ -3901,6 +3986,11 @@
           <t>77</t>
         </is>
       </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5A, 5B, 6A1, 6A-1, 6A2, 6A-2, 6B, 6C, 7</t>
+        </is>
+      </c>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
@@ -3908,6 +3998,11 @@
           <t>78</t>
         </is>
       </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
@@ -3915,6 +4010,11 @@
           <t>79</t>
         </is>
       </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
@@ -3922,6 +4022,11 @@
           <t>8</t>
         </is>
       </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
@@ -3929,6 +4034,11 @@
           <t>80</t>
         </is>
       </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
@@ -3936,6 +4046,11 @@
           <t>81</t>
         </is>
       </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
@@ -3943,6 +4058,11 @@
           <t>82</t>
         </is>
       </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
@@ -3950,6 +4070,11 @@
           <t>83</t>
         </is>
       </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
@@ -3957,6 +4082,11 @@
           <t>84</t>
         </is>
       </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
@@ -3964,6 +4094,11 @@
           <t>85</t>
         </is>
       </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
@@ -3971,6 +4106,11 @@
           <t>86</t>
         </is>
       </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
@@ -3978,6 +4118,11 @@
           <t>87</t>
         </is>
       </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
@@ -3985,6 +4130,11 @@
           <t>88</t>
         </is>
       </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
@@ -3992,6 +4142,11 @@
           <t>89</t>
         </is>
       </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
@@ -3999,6 +4154,11 @@
           <t>9</t>
         </is>
       </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 3</t>
+        </is>
+      </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
@@ -4006,6 +4166,11 @@
           <t>90</t>
         </is>
       </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
@@ -4013,6 +4178,11 @@
           <t>91</t>
         </is>
       </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
@@ -4020,6 +4190,11 @@
           <t>92</t>
         </is>
       </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
@@ -4027,6 +4202,11 @@
           <t>93</t>
         </is>
       </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
@@ -4034,6 +4214,11 @@
           <t>94</t>
         </is>
       </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
@@ -4041,6 +4226,11 @@
           <t>95</t>
         </is>
       </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
@@ -4048,6 +4238,11 @@
           <t>96</t>
         </is>
       </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
@@ -4055,6 +4250,11 @@
           <t>97</t>
         </is>
       </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
@@ -4062,11 +4262,21 @@
           <t>98</t>
         </is>
       </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
           <t>99</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>

</xml_diff>